<commit_message>
docs: close the weakest column in the rate transcription
The first verification round covered the columns unevenly. Sat-Overnight
was pinned by its $33.07 offset from 1-Day and Ground by its 1.05
increments, but 3-Day had nothing holding it except monotonicity — a
wrong digit there would have passed silently.

So From, Ground, 3-Day and 2-Day were read again from a fresh 9x render,
independently of the first pass, and diffed cell by cell: 136 cells, no
disagreement. Both readings are kept in the repo so the comparison can be
repeated.

Also records in the workbook's notes why the standard recalc did not run
(LibreOffice cannot open any file in this sandbox) and what replaced it.
Final state: 946 formula cells evaluated, no errors, and the only
verification failures are the two the FedEx source itself produces.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RFdtYaoBaVuFihSh1Mu5xS
</commit_message>
<xml_diff>
--- a/docs/data/fedex-shipping-rates.xlsx
+++ b/docs/data/fedex-shipping-rates.xlsx
@@ -4459,7 +4459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4500,106 +4500,130 @@
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>검증</t>
+          <t>검증 1차</t>
         </is>
       </c>
       <c r="B5" s="28" t="inlineStr">
         <is>
           <t>170칸 중 공란 3칸 제외 167개 값. Sat−1Day=$33.07 불변식이 34행 중 33행에서 성립, 전 열 단조 증가, 전 행 등급 순서 정상. Verification 시트에 수식으로 남김.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>검증 2차</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>1차 검사는 3-Day 컬럼을 단조성으로만 커버해 가장 약했음. 9배 렌더로 From·Ground·3-Day·2-Day를 1차와 별개로 다시 판독해 136셀 대조 — 불일치 0. 해당 컬럼 확정.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>확인 필요 1</t>
+          <t>수식 검증</t>
         </is>
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>Ground 요금 공란 — $37.00~$52.00, $52.00~$74.00, $74.00~$98.00 세 구간. 무료배송인지 Ground 미제공인지? (Danny)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>확인 필요 2</t>
-        </is>
-      </c>
-      <c r="B8" s="28" t="inlineStr">
-        <is>
-          <t>$894.00–$968.00 구간 Sat-Overnight = $870.94. 규칙대로면 $780.94. 원본 오타 의심. (FedEx/Danny)</t>
+          <t>942개 수식 셀 전체 평가, 오류 0. 파이썬 독립 계산과 표본 대조 일치. (LibreOffice가 이 환경에서 동작하지 않아 formulas 엔진으로 평가함)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
+          <t>확인 필요 1</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Ground 요금 공란 — $37.00~$52.00, $52.00~$74.00, $74.00~$98.00 세 구간. 무료배송인지 Ground 미제공인지? (Danny)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>확인 필요 2</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>$894.00–$968.00 구간 Sat-Overnight = $870.94. 규칙대로면 $780.94. 원본 오타 의심. (FedEx/Danny)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
           <t>확인 필요 3</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>구간 틈 2곳 — $98.00~$98.01, $521.00~$522.00. 경계 금액이 어느 구간인지. 이 파일은 'From ≤ 금액' 규칙으로 아래 구간에 흡수.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>확정</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>조회 기준 = 주문 subtotal (세금 전, 배송비 제외). Kai 확인 2026-09-10. 업그레이드 추가요금을 더해도 조회 구간이 바뀌지 않으므로 재계산 문제 없음.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>자동화 제외</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>NEXT DAY STANDARD / NEXT DAY EARLY 8:30AM — 원본에 'VARIES BY LOC.'로만 표기, 요금값 없음.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>조건부</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>SAT-OVERNIGHT — 원본 주석: 모든 도시에서 가능하지 않으니 결제 전 확인. Saturday 옵션은 금요일 Express 주문에만. Ground도 토요일 배송이 되는 경우가 있음.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>원본 주석</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Ground shipping is not a guaranteed service, but once "In transit", FEDEX guarantees the package will arrive by the ETA on their site. So, we cannot guarantee when the package will arrive before it ships out, but we can state, once UPS provides an ETA, they guarantee it will deliver by that time.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="39" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
+    <row r="18" ht="39" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>원본 주석</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>IMPORTANT NOTE: Saturday options is not available for all cities, please check before taking payment. Saturday Option is only available on Friday for Express orders. Ground shipping does deliver on Saturdays sometimes.</t>
         </is>

</xml_diff>